<commit_message>
Updated files by year
</commit_message>
<xml_diff>
--- a/files_by_year/2020_randomsample.xlsx
+++ b/files_by_year/2020_randomsample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,14 +16,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +48,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,96 +429,101 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R67"/>
+  <dimension ref="A1:S67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Published Date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Embargo Release</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>File Count</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>File 1</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>File 2</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>File 3</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>File 4</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>File 5</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>File 6</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>File 7</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>File 8</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>File 9</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>File 10</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>File 11</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>File 12</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>File 13</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
@@ -511,43 +532,43 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>xp68kg83m</t>
+          <t>v405s997r</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10.18130/v3-w8x8-4e63</t>
+          <t>10.18130/v3-kenp-ns95</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2020-05-11</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Ruddy_Blake_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-05</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>4</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ruddy_Blake_STS Research Paper.pdf</t>
+          <t>Osborne_Ben_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Ruddy_Blake_Sociotechnical Synthesis.pdf</t>
+          <t>Osborne_Ben_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Ruddy_Blake_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>Osborne_Ben_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Osborne_Ben_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
@@ -556,50 +577,53 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="n">
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>cz30pt14c</t>
+          <t>hm50ts32f</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10.18130/v3-sta0-dp73</t>
+          <t>10.18130/v3-04ne-6062</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2020-05-08</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Prospectus.pdf</t>
-        </is>
+          <t>2020-05-05</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>44321</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>STS Research Paper.pdf</t>
+          <t>Kleman_Davis_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Sociotechnical Synthesis.pdf</t>
+          <t>Kleman_Davis_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>Kleman_Davis_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Kleman_Davis_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
@@ -608,50 +632,53 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="n">
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>f7623d19j</t>
+          <t>1z40kt407</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.18130/v3-q10h-c192</t>
+          <t>10.18130/v3-ap0r-vb39</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>4</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Prospectus.pdf</t>
-        </is>
+          <t>2020-05-11</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>44146</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>STS Research Paper.pdf</t>
+          <t>Taylor_Jared_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Sociotechnical Synthesis.pdf</t>
+          <t>Taylor_Jared_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Technical Paper.pdf</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>Taylor_Jared_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Taylor_Jared_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
@@ -660,19 +687,20 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="n">
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2f75r8608</t>
+          <t>j38607499</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.18130/v3-2xg8-xt77</t>
+          <t>10.18130/v3-7w4q-5y18</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -680,30 +708,32 @@
           <t>2020-05-08</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Malcolm_Miller_Prospectus.pdf</t>
-        </is>
+      <c r="D5" s="2" t="n">
+        <v>45785</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Malcolm_Miller_STS Research Paper.pdf</t>
+          <t>Liu_Haotian_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Malcolm_Miller_Sociotechnical Synthesis.pdf</t>
+          <t>Liu_Haotian_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Malcolm_Miller_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>Liu_Haotian_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Liu_Haotian_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
@@ -712,50 +742,53 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="n">
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ft848r05s</t>
+          <t>0r967445n</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10.18130/v3-ekjh-yg77</t>
+          <t>10.18130/v3-fb4c-4206</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2020-04-28</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" t="inlineStr">
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>44143</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>Prospectus.pdf</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>STS Research Paper.pdf</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Sociotechnical Synthesis.pdf</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Technical Report.pdf</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
@@ -764,50 +797,53 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="n">
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3b591913n</t>
+          <t>wm117p61f</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.18130/v3-hw8f-ky52</t>
+          <t>10.18130/v3-hdvy-vw96</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2020-05-06</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>McGowan_Dillon_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>45785</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>McGowan_Dillon_STS Research Paper.pdf</t>
+          <t>Xiao_Sophia_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>McGowan_Dillon_Sociotechnical Synthesis.pdf</t>
+          <t>Xiao_Sophia_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>McGowan_Dillon_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
+          <t>Xiao_Sophia_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Xiao_Sophia_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
@@ -816,50 +852,51 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="n">
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>zk51vh45j</t>
+          <t>x920fx39s</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10.18130/v3-wsvj-4593</t>
+          <t>10.18130/v3-zadp-mp09</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Beck_Patrick_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-06</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>4</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Beck_Patrick_STS Research Paper.pdf</t>
+          <t>Prospectus.pdf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Beck_Patrick_Sociotechnical Synthesis.pdf</t>
+          <t>STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Beck_Patrick_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
+          <t>Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
@@ -868,50 +905,51 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="n">
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>vh53ww230</t>
+          <t>mw22v618w</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10.18130/v3-1efs-a793</t>
+          <t>10.18130/v3-t9gd-tn74</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2020-05-09</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>1_Qi_Zhouyang_Sociotechnical Synthesis.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>4</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2_Qi_Zhouyang_Technical Report.pdf</t>
+          <t>Rhodes_Carl_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3_Qi_Zhouyang_STS Research Paper.pdf</t>
+          <t>Rhodes_Carl_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>4_Qi_Zhouyang_Prospectus.pdf</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
+          <t>Rhodes_Carl_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Rhodes_Carl_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
@@ -920,50 +958,53 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="n">
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3197xm526</t>
+          <t>qb98mg195</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.18130/v3-vcz0-rz97</t>
+          <t>10.18130/v3-aqvg-ra59</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2020-05-06</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>1_Lithen_Brian_2020_BS.pdf</t>
-        </is>
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>45785</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2_Lithen_Brian_2020_BS.pdf</t>
+          <t>VazRapsoMendesdeAlmeida_Antonio_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3_Lithen_Brian_2020_BS.pdf</t>
+          <t>VazRapsoMendesdeAlmeida_Antonio_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>4_Lithen_Brian_2020_BS.pdf</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+          <t>VazRapsoMendesdeAlmeida_Antonio_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>VazRapsoMendesdeAlmeida_Antonio_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
@@ -972,50 +1013,53 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="n">
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9c67wn43v</t>
+          <t>5d86p096x</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.18130/v3-rpa5-t863</t>
+          <t>10.18130/v3-ty30-j864</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2020-05-07</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>4</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Goldman_Ari_Prospectus.pdf</t>
-        </is>
+          <t>2020-12-01</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>44531</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Goldman_Ari_STS_Research_Paper.pdf</t>
+          <t>Budzien_Liem_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Goldman_Ari_Sociotechnical_Synthesis.pdf</t>
+          <t>Budzien_Liem_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Goldman_Ari_Technical_Report.pdf</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr"/>
+          <t>Budzien_Liem_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Budzien_Liem_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
@@ -1024,50 +1068,51 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="n">
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>r781wg56f</t>
+          <t>c821gk39d</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.18130/v3-wjxs-6v02</t>
+          <t>10.18130/v3-40ae-bs76</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2020-05-07</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Craft_Nathaniel_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-05</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="n">
+        <v>4</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Craft_Nathaniel_STS Research Paper.pdf</t>
+          <t>Greene_Ian_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Craft_Nathaniel_Sociotechnical Synthesis.pdf</t>
+          <t>Greene_Ian_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Craft_Nathaniel_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
+          <t>Greene_Ian_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Greene_Ian_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
@@ -1076,50 +1121,53 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="n">
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>5h73pw64q</t>
+          <t>2z10wq84z</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.18130/v3-3j13-zh19</t>
+          <t>10.18130/v3-6cbm-7480</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2020-05-08</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>4</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Rosen_Zachary_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-05</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>45782</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Rosen_Zachary_STS Research Paper.pdf</t>
+          <t>Prater_Robert_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Rosen_Zachary_Sociotechnical Synthesis.pdf</t>
+          <t>Prater_Robert_STS_Research_Paper.pdf</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Rosen_Zachary_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
+          <t>Prater_Robert_Sociotechnical_Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Prater_Robert_Technical_Report.pdf</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
@@ -1128,50 +1176,53 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="n">
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>bv73c111t</t>
+          <t>st74cr269</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.18130/v3-fwht-wr32</t>
+          <t>10.18130/v3-czhr-y164</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2020-12-04</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Robb_Liam_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>44324</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Robb_Liam_STS Research Paper.pdf</t>
+          <t>Parodi_Victoria_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Robb_Liam_Sociotechnical Synthesis.pdf</t>
+          <t>Parodi_Victoria_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Robb_Liam_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
+          <t>Parodi_Victoria_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Parodi_Victoria_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
@@ -1180,50 +1231,51 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="n">
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>rn301205b</t>
+          <t>cr56n169n</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.18130/v3-4gnh-sn19</t>
+          <t>10.18130/v3-6p37-9h82</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2020-12-13</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>4</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Yoon_David_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-05</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="n">
+        <v>4</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Yoon_David_STS Research Paper.pdf</t>
+          <t>Lancaster_Anthony_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Yoon_David_Sociotechnical Synthesis.pdf</t>
+          <t>Lancaster_Anthony_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Yoon_David_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
+          <t>Lancaster_Anthony_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Lancaster_Anthony_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
@@ -1232,50 +1284,53 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="n">
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>g445cd873</t>
+          <t>7m01bm20j</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10.18130/v3-4c2q-m770</t>
+          <t>10.18130/v3-g2be-5b08</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2020-05-09</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>4</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Abazov_Renat_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>44143</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Abazov_Renat_STS Research Paper.pdf</t>
+          <t>Applegate_Dalton_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Abazov_Renat_Sociotechnical Synthesis.pdf</t>
+          <t>Applegate_Dalton_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Abazov_Renat_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
+          <t>Applegate_Dalton_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Applegate_Dalton_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
@@ -1284,50 +1339,51 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="n">
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>n009w279z</t>
+          <t>2514nm19s</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10.18130/v3-6cf5-xb11</t>
+          <t>10.18130/v3-hvj6-j702</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2020-05-07</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>4</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Nguyen_John_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-06</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>4</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Nguyen_John_STS Research Paper.pdf</t>
+          <t>1_Bennett_David_2020_BS_STS_Research_Paper.pdf</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Nguyen_John_Sociotechnical Synthesis.pdf</t>
+          <t>2_Bennett_David_2020_BS_Technical_Report.pdf</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Nguyen_John_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr"/>
+          <t>3_Bennett_David_2020_BS_Sociotechnical_Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>4_Bennett_David_2020_BS_Prospectus.pdf</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
@@ -1336,50 +1392,53 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="n">
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>fb494910k</t>
+          <t>ff365589s</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10.18130/v3-0pp1-gv81</t>
+          <t>10.18130/v3-pavj-mx77</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2020-05-07</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Nathan_Jeremy_Prospectus</t>
-        </is>
+          <t>2020-05-11</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>44146</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Nathan_Jeremy_STS Research Paper.pdf</t>
+          <t>Hays_Philip_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Nathan_Jeremy_Sociotechnical Synthesis.pdf</t>
+          <t>Hays_Philip_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Nathan_Jeremy_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
+          <t>Hays_Philip_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Hays_Philip_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
@@ -1388,50 +1447,53 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="n">
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>gt54kn73k</t>
+          <t>pr76f403n</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10.18130/v3-va2v-ps29</t>
+          <t>10.18130/v3-wpe4-es14</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2020-12-03</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>4</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Prospectus.pdf</t>
-        </is>
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>44143</v>
+      </c>
+      <c r="E19" t="n">
+        <v>4</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>STS Research Paper.pdf</t>
+          <t>Plutchak_Spencer_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Sociotechnical Synthesis.pdf</t>
+          <t>Plutchak_Spencer_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr"/>
+          <t>Plutchak_Spencer_Sociotechnical_Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Plutchak_Spencer_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
@@ -1440,50 +1502,53 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="n">
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>bv73c1123</t>
+          <t>t435gd71z</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.18130/v3-gz46-gf15</t>
+          <t>10.18130/v3-c1ck-pt91</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2020-12-15</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Blankinship_Thomas_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>44324</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Blankinship_Thomas_STS Research Paper.pdf</t>
+          <t>Kamali_Rojeen_Design and Development of a Kinetic Power Pack.pdf</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Blankinship_Thomas_Sociotechnical Synthesis.pdf</t>
+          <t>Kamali_Rojeen_Prospectus.pdf</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Blankinship_Thomas_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
+          <t>Kamali_Rojeen_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Kamali_Rojeen_The Rise of Social Media Leaving Its Trace on National Parks.pdf</t>
+        </is>
+      </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
@@ -1492,19 +1557,20 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="n">
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2514nm20j</t>
+          <t>ff365585p</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10.18130/v3-abrg-3y32</t>
+          <t>10.18130/v3-tfca-1274</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1512,30 +1578,32 @@
           <t>2020-05-08</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>4</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>O'Hanlon_Michael_Prospectus.pdf</t>
-        </is>
+      <c r="D21" s="2" t="n">
+        <v>45785</v>
+      </c>
+      <c r="E21" t="n">
+        <v>4</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>O'Hanlon_Michael_STS Research Paper.pdf</t>
+          <t>Smith_Henry_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>O'Hanlon_Michael_Sociotechnical Synthesis.pdf</t>
+          <t>Smith_Henry_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>O'Hanlon_Michael_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
+          <t>Smith_Henry_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Smith_Henry_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
@@ -1544,19 +1612,20 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="n">
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>bn9997412</t>
+          <t>sn009z36t</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10.18130/v3-4v83-4c35</t>
+          <t>10.18130/v3-5kbm-8737</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1564,30 +1633,32 @@
           <t>2020-05-07</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>4</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Santana_Joshua_Prospectus.pdf</t>
-        </is>
+      <c r="D22" s="2" t="n">
+        <v>44324</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Santana_Joshua_STS Research Paper.pdf</t>
+          <t>Nelson_Joseph_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Santana_Joshua_Sociotechnical Synthesis.pdf</t>
+          <t>Nelson_Joseph_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Santana_Joshua_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
+          <t>Nelson_Joseph_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Nelson_Joseph_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
@@ -1596,50 +1667,53 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="n">
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4m90dw08z</t>
+          <t>1r66j167b</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10.18130/v3-va15-2393</t>
+          <t>10.18130/v3-naed-m848</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2020-05-01</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>4</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Prospectus.pdf</t>
-        </is>
+          <t>2020-05-06</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>45783</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>STS Research Paper.pdf</t>
+          <t>Sitoula_Yukesh_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Sociotechnical Synthesis.pdf</t>
+          <t>Sitoula_Yukesh_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
+          <t>Sitoula_Yukesh_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Sitoula_Yukesh_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
@@ -1648,50 +1722,53 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="n">
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>9z903052f</t>
+          <t>rb68xc65x</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10.18130/v3-mefg-h820</t>
+          <t>10.18130/v3-a2jk-7w73</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>4</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Mackenzie_Georgia_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-09</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>44325</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Mackenzie_Georgia_STS Research Paper.pdf</t>
+          <t>Cave_Samuel_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Mackenzie_Georgia_Sociotechnical Synthesis.pdf</t>
+          <t>Cave_Samuel_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Mackenzie_Georgia_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
+          <t>Cave_Samuel_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Cave_Samuel_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
@@ -1700,50 +1777,53 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="n">
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>hx11xf99m</t>
+          <t>w9505105g</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10.18130/v3-8z7x-y730</t>
+          <t>10.18130/v3-aac2-fm63</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2020-05-08</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>4</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Zeng_Zi_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>44142</v>
+      </c>
+      <c r="E25" t="n">
+        <v>4</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Zeng_Zi_STS Research Paper.pdf</t>
+          <t>Han_Chris_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Zeng_Zi_Sociotechnical Synthesis.pdf</t>
+          <t>Han_Chris_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Zeng_Zi_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr"/>
+          <t>Han_Chris_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Han_Chris_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
@@ -1752,50 +1832,53 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="n">
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>hm50ts32f</t>
+          <t>mc87pq87t</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>10.18130/v3-04ne-6062</t>
+          <t>10.18130/v3-jgns-s519</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>4</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Kleman_Davis_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>44142</v>
+      </c>
+      <c r="E26" t="n">
+        <v>4</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Kleman_Davis_STS Research Paper.pdf</t>
+          <t>Hecht_Samuel_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Kleman_Davis_Sociotechnical Synthesis.pdf</t>
+          <t>Hecht_Samuel_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Kleman_Davis_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
+          <t>Hecht_Samuel_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Hecht_Samuel_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
@@ -1804,50 +1887,51 @@
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="n">
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>w9505103x</t>
+          <t>q524jp338</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10.18130/v3-m3yz-yk33</t>
+          <t>10.18130/v3-jae0-s904</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2020-04-27</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>4</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Prospectus.pdf</t>
-        </is>
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>4</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>STS Research Paper.pdf</t>
+          <t>Dawkins_Quinlan_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Sociotechnical Synthesis.pdf</t>
+          <t>Dawkins_Quinlan_STS_Research.pdf</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr"/>
+          <t>Dawkins_Quinlan_Technical_Report.pdf</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Dawkins_Quinlan_Title_Page_and_Sociotechnical_Synthesis.pdf</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
@@ -1856,50 +1940,53 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="n">
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>44558d93g</t>
+          <t>qf85nb89w</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10.18130/v3-jh4p-vn08</t>
+          <t>10.18130/v3-4mty-6n32</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>4</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Martin_Zachry_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>45784</v>
+      </c>
+      <c r="E28" t="n">
+        <v>4</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Martin_Zachry_STS Research Paper.pdf</t>
+          <t>Peters_Dylan_Contextual_Analysis_of_Technology_Use_in_Resource_Challenged_Schools.pdf</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Martin_Zachry_Sociotechnical Synthesis.pdf</t>
+          <t>Peters_Dylan_Prospectus.pdf</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Martin_Zachry_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
+          <t>Peters_Dylan_Raising_Deforestation_Awareness_Through_Online_Education.pdf</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Peters_Dylan_Sociotechnical_Synthesis.pdf</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
@@ -1908,50 +1995,53 @@
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="n">
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>gh93h0127</t>
+          <t>j6731427h</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10.18130/v3-zzkc-te53</t>
+          <t>10.18130/v3-y1ce-3k41</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>4</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>1_De_Luis_2020_BS.pdf</t>
-        </is>
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>44143</v>
+      </c>
+      <c r="E29" t="n">
+        <v>4</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2_De_Luis_2020_BS.pdf</t>
+          <t>Wood_Michael_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>3_De_Luis_2020_BS.pdf</t>
+          <t>Wood_Michael_STS_Research_Paper.pdf</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>4_De_Luis_2020_BS.pdf</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr"/>
+          <t>Wood_Michael_Sociotechnical_Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Wood_Michael_Technical_Report.pdf</t>
+        </is>
+      </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
@@ -1960,50 +2050,51 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="n">
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>v692t6855</t>
+          <t>mp48sd28n</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10.18130/v3-5kx4-yx65</t>
+          <t>10.18130/v3-kdq2-1w37</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>4</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Beaubien_Allyson_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-04</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>4</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Beaubien_Allyson_STS Research Paper.pdf</t>
+          <t>Carroll_Kaelyn_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Beaubien_Allyson_Sociotechnical Synthesis.pdf</t>
+          <t>Carroll_Kaelyn_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Beaubien_Allyson_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr"/>
+          <t>Carroll_Kaelyn_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Carroll_Kaelyn_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
@@ -2012,19 +2103,20 @@
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="n">
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>sq87bv18c</t>
+          <t>h989r392b</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10.18130/v3-b2qj-yw49</t>
+          <t>10.18130/v3-qh84-xp65</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2032,30 +2124,30 @@
           <t>2020-05-07</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>4</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Awasthi_Rohni_Design_Optimization_of_an_Ergonomic_Lead_Garment.pdf</t>
-        </is>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>4</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Awasthi_Rohni_Prospectus.pdf</t>
+          <t>Oxford_Andrew_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Awasthi_Rohni_Sociotechnical_Synthesis.pdf</t>
+          <t>Oxford_Andrew_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Awasthi_Rohni_The_Impact_of_Legislation_on_the_Medical_Device_Industry.pdf</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr"/>
+          <t>Oxford_Andrew_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Oxford_Andrew_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
@@ -2064,50 +2156,53 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="n">
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>dr26xz215</t>
+          <t>9g54xj191</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>10.18130/v3-8mpf-jp48</t>
+          <t>10.18130/v3-0sj3-bv64</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2020-05-07</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>4</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>1_Burbach_Eric_2020_BS.pdf</t>
-        </is>
+          <t>2020-04-30</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>44316</v>
+      </c>
+      <c r="E32" t="n">
+        <v>4</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2_Burbach_Eric_2020_BS.pdf</t>
+          <t>Prospectus.pdf</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>3_Burbach_Eric_2020_BS.pdf</t>
+          <t>STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>4_Burbach_Eric_2020_BS.pdf</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr"/>
+          <t>Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
@@ -2116,50 +2211,53 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="n">
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3t945r28b</t>
+          <t>5x21tg04h</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10.18130/v3-mbsr-vp62</t>
+          <t>10.18130/v3-0p6h-gh50</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2020-05-08</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>4</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Umansky_Hannah_Clean_Air_How_Policy_and_Data_Can_Enforce_Human_Rights.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>45784</v>
+      </c>
+      <c r="E33" t="n">
+        <v>4</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Umansky_Hannah_High_Resolution_Satellite_Imaging_of_Nitrogen_Dioxide_from_Low_Earth_Orbit.pdf</t>
+          <t>Lansing_Maryanna_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Umansky_Hannah_Prospectus.pdf</t>
+          <t>Lansing_Maryanna_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Umansky_Hannah_Sociotechnical_Synthesis.pdf</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr"/>
+          <t>Lansing_Maryanna_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Lansing_Maryanna_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
@@ -2168,50 +2266,51 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="n">
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>rn301187m</t>
+          <t>cf95jc084</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>10.18130/v3-qtvp-n205</t>
+          <t>10.18130/v3-f8zb-pw68</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2020-05-01</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>4</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>DuCharme_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-06</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>4</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>DuCharme_STS_Research_Paper.pdf</t>
+          <t>Shiu_Michael_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>DuCharme_SocioTechnical_Synthesis.pdf</t>
+          <t>Shiu_Michael_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>DuCharme_Technical_Report.pdf</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
+          <t>Shiu_Michael_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Shiu_Michael_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
@@ -2220,50 +2319,53 @@
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="n">
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>7m01bm24n</t>
+          <t>3n203z68k</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>10.18130/v3-p0y4-xn04</t>
+          <t>10.18130/v3-ejcp-et79</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>4</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Hisiro_Wade_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>44689</v>
+      </c>
+      <c r="E35" t="n">
+        <v>4</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Hisiro_Wade_STS Research Paper.pdf</t>
+          <t>Medina_Joseff_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Hisiro_Wade_Sociotechnical Synthesis.pdf</t>
+          <t>Medina_Joseff_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Hisiro_Wade_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr"/>
+          <t>Medina_Joseff_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Medina_Joseff_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
@@ -2272,50 +2374,53 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="n">
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5138jf445</t>
+          <t>gb19f651g</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>10.18130/v3-1e6n-3657</t>
+          <t>10.18130/v3-zda1-ys92</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2020-05-04</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>4</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Handy_Alec_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-06</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>45783</v>
+      </c>
+      <c r="E36" t="n">
+        <v>4</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Handy_Alec_STS_Research_Paper.pdf</t>
+          <t>Goldrich_Madison_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Handy_Alec_Sociotechnical_Synthesis.pdf</t>
+          <t>Goldrich_Madison_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Handy_Alec_Technical_Report.pdf</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr"/>
+          <t>Goldrich_Madison_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Goldrich_Madison_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
@@ -2324,50 +2429,53 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="n">
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2z10wq82d</t>
+          <t>nz8060305</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>10.18130/v3-jwc2-dd97</t>
+          <t>10.18130/v3-j5ny-b960</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2020-05-01</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>4</v>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Alok_Akanksha_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>45785</v>
+      </c>
+      <c r="E37" t="n">
+        <v>4</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Alok_Akanksha_STS Research Paper.pdf</t>
+          <t>Mahaffey_Brad_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Alok_Akanksha_Sociotechnical Synthesis.pdf</t>
+          <t>Mahaffey_Brad_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Alok_Akanksha_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr"/>
+          <t>Mahaffey_Brad_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Mahaffey_Brad_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
@@ -2376,51 +2484,58 @@
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="n">
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>05741s34c</t>
+          <t>kp78gh18r</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10.18130/v3-nd0c-6s14</t>
+          <t>10.18130/v3-g150-1m96</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2020-05-07</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>4</v>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Pazhwak_Bobby_Prospectus.pdf</t>
-        </is>
+          <t>2020-12-03</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>45994</v>
+      </c>
+      <c r="E38" t="n">
+        <v>5</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Pazhwak_Bobby_STS Research Paper.pdf</t>
+          <t>Kristian Johnson - Prospectus.pdf</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Pazhwak_Bobby_Sociotechnical Synthesis.pdf</t>
+          <t>Kristian Johnson - STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Pazhwak_Bobby_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
+          <t>Kristian Johnson - Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Kristian Johnson - Technical Report.pdf</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Kristian Johnson - Thesis Title Page.pdf</t>
+        </is>
+      </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
@@ -2428,50 +2543,53 @@
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="n">
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5d86p092t</t>
+          <t>xg94hq24w</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10.18130/v3-vf8y-5320</t>
+          <t>10.18130/v3-yj9y-n451</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2020-05-11</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>4</v>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Sheng_Yuelan_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-06</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>45783</v>
+      </c>
+      <c r="E39" t="n">
+        <v>4</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sheng_Yuelan_STS Research Paper.pdf</t>
+          <t>Rashid_Nushaba_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Sheng_Yuelan_Sociotechnical Synthesis.pdf</t>
+          <t>Rashid_Nushaba_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Sheng_Yuelan_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr"/>
+          <t>Rashid_Nushaba_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Rashid_Nushaba_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
@@ -2480,50 +2598,53 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="n">
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>4b29b6449</t>
+          <t>1831ck50n</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10.18130/v3-xwk8-9f44</t>
+          <t>10.18130/v3-70qt-2k25</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>4</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Page_Brady_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-06</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>45783</v>
+      </c>
+      <c r="E40" t="n">
+        <v>4</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Page_Brady_STS_Research_Paper.pdf</t>
+          <t>DeWoody_Jillian_A COST TO CONVENIENCE: HOW CONSUMERS MANAGE PRIVACY VALUES ONLINE.pdf</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Page_Brady_Sociotechnical_Synthesis.pdf</t>
+          <t>DeWoody_Jillian_CONNECTING AT-HOME NURSES WITH PATIENTS ONLINE.pdf</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Page_Brady_Technical_Report.pdf</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr"/>
+          <t>DeWoody_Jillian_Prospectus.pdf</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DeWoody_Jillian_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
@@ -2532,50 +2653,51 @@
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="n">
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>xk81jk90h</t>
+          <t>tq57nr580</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10.18130/v3-pwk1-kf79</t>
+          <t>10.18130/v3-k1ky-bd18</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2020-05-07</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>4</v>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Rohrer_Kelly_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-05</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="n">
+        <v>4</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Rohrer_Kelly_STS Research Paper.pdf</t>
+          <t>Nguyen_Judy_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Rohrer_Kelly_Sociotechnical Synthesis.pdf</t>
+          <t>Nguyen_Judy_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Rohrer_Kelly_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr"/>
+          <t>Nguyen_Judy_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Nguyen_Judy_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
@@ -2584,50 +2706,53 @@
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="n">
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1831ck47b</t>
+          <t>nk322d88c</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>10.18130/v3-gxb0-vc63</t>
+          <t>10.18130/v3-zmjr-0x25</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2020-04-29</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>4</v>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Prospectus.pdf</t>
-        </is>
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>45786</v>
+      </c>
+      <c r="E42" t="n">
+        <v>4</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>STS Research Paper.pdf</t>
+          <t>Johnson_Johannes_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Sociotechnical Synthesis.pdf</t>
+          <t>Johnson_Johannes_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr"/>
+          <t>Johnson_Johannes_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Johnson_Johannes_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
@@ -2636,50 +2761,53 @@
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="n">
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>h989r394w</t>
+          <t>bn9997412</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>10.18130/v3-h8zq-qa34</t>
+          <t>10.18130/v3-4v83-4c35</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2020-05-08</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>4</v>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Ramirez_Jonathan_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>44142</v>
+      </c>
+      <c r="E43" t="n">
+        <v>4</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Ramirez_Jonathan_STS Research Paper.pdf</t>
+          <t>Santana_Joshua_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Ramirez_Jonathan_Sociotechnical Synthesis.pdf</t>
+          <t>Santana_Joshua_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Ramirez_Jonathan_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr"/>
+          <t>Santana_Joshua_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Santana_Joshua_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
@@ -2688,50 +2816,53 @@
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="n">
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>37720d42k</t>
+          <t>t148fh895</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>10.18130/v3-0stj-1t96</t>
+          <t>10.18130/v3-45wh-z470</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>4</v>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Geerdes_Nathaniel_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>45785</v>
+      </c>
+      <c r="E44" t="n">
+        <v>4</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Geerdes_Nathaniel_STS_Research_Paper.pdf</t>
+          <t>Park_Nathan_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Geerdes_Nathaniel_Sociotechnical_Synthesis.pdf</t>
+          <t>Park_Nathan_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Geerdes_Nathaniel_Technical_Report.pdf</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr"/>
+          <t>Park_Nathan_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Park_Nathan_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
@@ -2740,50 +2871,51 @@
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="n">
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>q524jp35t</t>
+          <t>9019s3032</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>10.18130/v3-cncd-yx23</t>
+          <t>10.18130/v3-jsmn-1n88</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>4</v>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Prospectus.pdf</t>
-        </is>
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="n">
+        <v>4</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>STS Research Paper.pdf</t>
+          <t>1_Blibo_Nia_2020_BS.pdf</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Sociotechnical Synthesis.pdf</t>
+          <t>2_Blibo_Nia_2020_BS.pdf</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr"/>
+          <t>3_Blibo_Nia_2020_BS.pdf</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>4_Blibo_Nia_2020_BS.pdf</t>
+        </is>
+      </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
@@ -2792,50 +2924,53 @@
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="n">
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>6m311p740</t>
+          <t>z603qx948</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>10.18130/v3-f7tk-9s68</t>
+          <t>10.18130/v3-v9xz-k347</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
-        <v>4</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>1_Rowe_Charles_SocioTechnical_Synthesis_2020_BS.pdf</t>
-        </is>
+          <t>2020-05-03</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>45780</v>
+      </c>
+      <c r="E46" t="n">
+        <v>4</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2_Rowe_Charles_Technical_Report_2020_BS.pdf</t>
+          <t>Stenberg_Sabrina_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>3_Rowe_Charles_STS_Research_Paper_2020_BS.pdf</t>
+          <t>Stenberg_Sabrina_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>4_Rowe_Charles_Prospectus_2020_BS.pdf</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr"/>
+          <t>Stenberg_Sabrina_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Stenberg_Sabrina_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
@@ -2844,50 +2979,51 @@
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="n">
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>mk61rh57k</t>
+          <t>12579s883</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>10.18130/v3-3r04-tm69</t>
+          <t>10.18130/v3-xab9-2m43</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2020-05-08</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>4</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Kosolwattana_Tanapol_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-04</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="n">
+        <v>4</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Kosolwattana_Tanapol_STS Research Paper.pdf</t>
+          <t>1_Yun_James_2020_BS_Sociotechnical_Synthesis.pdf</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Kosolwattana_Tanapol_Sociotechnical Synthesis.pdf</t>
+          <t>2_Yun_James_2020_BS_Technical_Report.pdf</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Kosolwattana_Tanapol_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr"/>
+          <t>3_Yun_James_2020_BS_STS_Research_Paper.pdf</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>4_Yun_James_2020_BS_Prospectus.pdf</t>
+        </is>
+      </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
@@ -2896,50 +3032,53 @@
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="n">
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>d504rk84n</t>
+          <t>5999n4045</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>10.18130/v3-vqhv-9a55</t>
+          <t>10.18130/v3-4qv8-ew91</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2020-05-01</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>4</v>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>1_Vallar_Frederic_2020_BS_Sociotechnical_Synthesis.pdf</t>
-        </is>
+          <t>2020-05-04</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>44320</v>
+      </c>
+      <c r="E48" t="n">
+        <v>4</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2_Vallar_Frederic_2020_BS_Technical_Report.pdf</t>
+          <t>Saint-Jean_Edler_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>3_Vallar_Frederic_2020_BS_STS_Research_Paper.pdf</t>
+          <t>Saint-Jean_Edler_STS_Research_Paper.pdf</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>4_Vallar_Frederic_2020_BS_Prospectus.pdf</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr"/>
+          <t>Saint-Jean_Edler_Sociotechnical_Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Saint-Jean_Edler_Technical_Report.pdf</t>
+        </is>
+      </c>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
@@ -2948,50 +3087,51 @@
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="n">
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>xp68kg74n</t>
+          <t>v118rf289</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>10.18130/v3-pqrd-jq22</t>
+          <t>10.18130/v3-2mek-tm13</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2020-05-07</t>
-        </is>
-      </c>
-      <c r="D49" t="n">
-        <v>4</v>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Riedy_Julia_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-05</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="n">
+        <v>4</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Riedy_Julia_STS Research Paper.pdf</t>
+          <t>Gerken_Jeffrey_STS Research_Paper.pdf</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Riedy_Julia_Sociotechnical Synthesis.pdf</t>
+          <t>Gerken_Jeffrey_Sociotechnical_Synthesis.pdf</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Riedy_Julia_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr"/>
+          <t>Gerken_Jeffrey_Technical_Report.pdf</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Gerken_Jeffrey__Prospectus.pdf</t>
+        </is>
+      </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
@@ -3000,50 +3140,53 @@
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="n">
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>8k71nh65h</t>
+          <t>tq57nr57q</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>10.18130/v3-t4wg-z103</t>
+          <t>10.18130/v3-d6z5-7c30</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2020-04-29</t>
-        </is>
-      </c>
-      <c r="D50" t="n">
-        <v>4</v>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Prospectus.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>44688</v>
+      </c>
+      <c r="E50" t="n">
+        <v>4</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>STS Research Paper.pdf</t>
+          <t>Ahi_Termeh_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Sociotechnical Synthesis.pdf</t>
+          <t>Ahi_Termeh_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr"/>
+          <t>Ahi_Termeh_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Ahi_Termeh_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
@@ -3052,50 +3195,53 @@
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="n">
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>d504rk87g</t>
+          <t>kk91fm098</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>10.18130/v3-6ftk-p152</t>
+          <t>10.18130/v3-ft9y-ns45</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2020-05-07</t>
-        </is>
-      </c>
-      <c r="D51" t="n">
-        <v>4</v>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Nelson_Sarah_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-04</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>44320</v>
+      </c>
+      <c r="E51" t="n">
+        <v>4</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Nelson_Sarah_STS Research Paper.pdf</t>
+          <t>Hu_Jinming_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Nelson_Sarah_Sociotechnical Synthesis.pdf</t>
+          <t>Hu_Jinming_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Nelson_Sarah_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr"/>
+          <t>Hu_Jinming_Socialtechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Hu_Jinming_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
@@ -3104,19 +3250,20 @@
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="n">
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>th83kz918</t>
+          <t>k35694820</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>10.18130/v3-465k-1k60</t>
+          <t>10.18130/v3-jkrr-h587</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3124,30 +3271,30 @@
           <t>2020-05-05</t>
         </is>
       </c>
-      <c r="D52" t="n">
-        <v>4</v>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Nathan_SarahWinston_Prospectus.pdf</t>
-        </is>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="n">
+        <v>4</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Nathan_SarahWinston_STS Research Paper.pdf</t>
+          <t>Prospectus.pdf</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Nathan_SarahWinston_Sociotechnical Synthesis.pdf</t>
+          <t>STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Nathan_SarahWinston_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr"/>
+          <t>Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
@@ -3156,50 +3303,53 @@
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="n">
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>9c67wn401</t>
+          <t>vh53ww39w</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>10.18130/v3-ywke-3t09</t>
+          <t>10.18130/v3-28z2-9n98</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2020-05-09</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>4</v>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Tahir_Amna_Prospectus.pdf</t>
-        </is>
+          <t>2020-12-04</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>44535</v>
+      </c>
+      <c r="E53" t="n">
+        <v>4</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Tahir_Amna_STS_Research_Paper.pdf</t>
+          <t>Clark_David_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Tahir_Amna_Sociotechnical_Synthesis.pdf</t>
+          <t>Clark_David_STS_Research_Paper.pdf</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Tahir_Amna_Technical_Report.pdf</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr"/>
+          <t>Clark_David_Sociotechnical_Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Clark_David_Technical_Report.pdf</t>
+        </is>
+      </c>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
@@ -3208,50 +3358,53 @@
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr"/>
       <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="n">
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2514nm19s</t>
+          <t>fb494910k</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>10.18130/v3-hvj6-j702</t>
+          <t>10.18130/v3-0pp1-gv81</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2020-05-06</t>
-        </is>
-      </c>
-      <c r="D54" t="n">
-        <v>4</v>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>1_Bennett_David_2020_BS_STS_Research_Paper.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>45785</v>
+      </c>
+      <c r="E54" t="n">
+        <v>4</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2_Bennett_David_2020_BS_Technical_Report.pdf</t>
+          <t>Nathan_Jeremy_Prospectus</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>3_Bennett_David_2020_BS_Sociotechnical_Synthesis.pdf</t>
+          <t>Nathan_Jeremy_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>4_Bennett_David_2020_BS_Prospectus.pdf</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr"/>
+          <t>Nathan_Jeremy_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Nathan_Jeremy_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
@@ -3260,50 +3413,51 @@
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr"/>
-      <c r="R54" t="n">
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>n870zr36p</t>
+          <t>3484zh40n</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>10.18130/v3-1xch-sw36</t>
+          <t>10.18130/v3-p8z8-3564</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2020-05-06</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
-        <v>4</v>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>STS Prospectus.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="n">
+        <v>4</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>STS Research Paper.pdf</t>
+          <t>1_ODonnell_Ian_2020_BS.pdf</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Sociotechnical Synthesis.pdf</t>
+          <t>2_ODonnell_Ian_2020_BS.pdf</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr"/>
+          <t>3_ODonnell_Ian_2020_BS.pdf</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>4_ODonnell_Ian_2020_BS.pdf</t>
+        </is>
+      </c>
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
@@ -3312,50 +3466,53 @@
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr"/>
       <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="n">
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>c821gk39d</t>
+          <t>kw52j8555</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>10.18130/v3-40ae-bs76</t>
+          <t>10.18130/v3-r28e-pb08</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D56" t="n">
-        <v>4</v>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Greene_Ian_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>44323</v>
+      </c>
+      <c r="E56" t="n">
+        <v>4</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Greene_Ian_STS Research Paper.pdf</t>
+          <t>Thiringer_Stephen_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Greene_Ian_Sociotechnical Synthesis.pdf</t>
+          <t>Thiringer_Stephen_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Greene_Ian_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr"/>
+          <t>Thiringer_Stephen_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Thiringer_Stephen_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
@@ -3364,50 +3521,51 @@
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr"/>
       <c r="Q56" t="inlineStr"/>
-      <c r="R56" t="n">
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>zp38wd13s</t>
+          <t>x920fx43c</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>10.18130/v3-fbkg-ty09</t>
+          <t>10.18130/v3-c2k6-as26</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2020-05-07</t>
-        </is>
-      </c>
-      <c r="D57" t="n">
-        <v>4</v>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Woloff_Jason_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-08</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="n">
+        <v>4</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Woloff_Jason_STS Research Paper.pdf</t>
+          <t>ONeill_Noah_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Woloff_Jason_Sociotechnical Synthesis.pdf</t>
+          <t>ONeill_Noah_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Woloff_Jason_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr"/>
+          <t>ONeill_Noah_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>ONeill_Noah_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
@@ -3416,50 +3574,51 @@
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr"/>
       <c r="Q57" t="inlineStr"/>
-      <c r="R57" t="n">
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>nz806027v</t>
+          <t>44558d93g</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10.18130/v3-4sqp-nv06</t>
+          <t>10.18130/v3-jh4p-vn08</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2020-05-07</t>
-        </is>
-      </c>
-      <c r="D58" t="n">
-        <v>4</v>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Perry_Lauren_Adaptive Mobile Sensing: Leveraging Machine Learning for Efficient Human Behavior Modeling.pdf</t>
-        </is>
+          <t>2020-05-05</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="n">
+        <v>4</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Perry_Lauren_Examining Data Privacy Regulation to Protect Personal Health Records.pdf</t>
+          <t>Martin_Zachry_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Perry_Lauren_Prospectus.pdf</t>
+          <t>Martin_Zachry_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Perry_Lauren_Sociotechnical Synthesis.pdf</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr"/>
+          <t>Martin_Zachry_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Martin_Zachry_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
@@ -3468,19 +3627,20 @@
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr"/>
       <c r="Q58" t="inlineStr"/>
-      <c r="R58" t="n">
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>zw12z5973</t>
+          <t>zs25x8959</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>10.18130/v3-awcr-qn60</t>
+          <t>10.18130/v3-ew8g-tz70</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3488,30 +3648,30 @@
           <t>2020-05-08</t>
         </is>
       </c>
-      <c r="D59" t="n">
-        <v>4</v>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>1_Karamete_Tan_2020_BS.pdf</t>
-        </is>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="n">
+        <v>4</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2_Karamete_Tan_2020_BS.pdf</t>
+          <t>Prospectus.pdf</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>3_Karamete_Tan_2020_BS.pdf</t>
+          <t>STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>4_Karamete_Tan_2020_BS.pdf</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr"/>
+          <t>Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr"/>
@@ -3520,50 +3680,53 @@
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr"/>
       <c r="Q59" t="inlineStr"/>
-      <c r="R59" t="n">
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>02870w46x</t>
+          <t>736665352</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>10.18130/v3-qjs0-k505</t>
+          <t>10.18130/v3-f0qv-xg44</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2020-05-06</t>
-        </is>
-      </c>
-      <c r="D60" t="n">
-        <v>4</v>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Metzger_Benjamin_Prospectus.pdf</t>
-        </is>
+          <t>2020-12-12</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>46004</v>
+      </c>
+      <c r="E60" t="n">
+        <v>4</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Metzger_Benjamin_STS Research Paper.pdf</t>
+          <t>Alvarado_Manuel_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Metzger_Benjamin_Sociotechnical Synthesis.pdf</t>
+          <t>Alvarado_Manuel_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Metzger_Benjamin_Thesis</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr"/>
+          <t>Alvarado_Manuel_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Alvarado_Manuel_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr"/>
@@ -3572,50 +3735,51 @@
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr"/>
       <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="n">
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>sn009z41p</t>
+          <t>h702q701m</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>10.18130/v3-4qkh-s139</t>
+          <t>10.18130/v3-tf8b-bd61</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D61" t="n">
-        <v>4</v>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Long_Jane_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="n">
+        <v>4</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Long_Jane_STS Research Paper.pdf</t>
+          <t>Farruggio_Andrew_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Long_Jane_Sociotechnical Synthesis.pdf</t>
+          <t>Farruggio_Andrew_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Long_Jane_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr"/>
+          <t>Farruggio_Andrew_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Farruggio_Andrew_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>
@@ -3624,50 +3788,51 @@
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr"/>
       <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="n">
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>qz20st15d</t>
+          <t>b8515n95w</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>10.18130/v3-5mtj-bt32</t>
+          <t>10.18130/v3-26sx-4150</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
-        </is>
-      </c>
-      <c r="D62" t="n">
-        <v>4</v>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Chandra_Aniket_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-11</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="n">
+        <v>4</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Chandra_Aniket_STS_Research_Paper.pdf</t>
+          <t>1_Hanrahan_Garrett_2020_BS.pdf</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Chandra_Aniket_Sociotechnical_Synthesis.pdf</t>
+          <t>2_Hanrahan_Garrett_2020_BS.pdf</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Chandra_Aniket_Technical_Report.pdf</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr"/>
+          <t>3_Hanrahan_Garrett_2020_BS.pdf</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>4_Hanrahan_Garrett_2020_BS.pdf</t>
+        </is>
+      </c>
       <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr"/>
@@ -3676,19 +3841,20 @@
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr"/>
       <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="n">
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>h702q694d</t>
+          <t>3t945r31n</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>10.18130/v3-mk3x-4k40</t>
+          <t>10.18130/v3-1wwy-bn80</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3696,30 +3862,32 @@
           <t>2020-05-07</t>
         </is>
       </c>
-      <c r="D63" t="n">
-        <v>4</v>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Prospectus Title Page_Prospectus.pdf</t>
-        </is>
+      <c r="D63" s="2" t="n">
+        <v>44142</v>
+      </c>
+      <c r="E63" t="n">
+        <v>4</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>STS Title Page_STS Research Paper.pdf</t>
+          <t>Radhakrishnan_Keerthi_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Technical Title Page_CapstoneTechnical Report.pdf</t>
+          <t>Radhakrishnan_Keerthi_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Thesis Title Page_Sociotechnical Synthesis_Table of Contents.pdf</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr"/>
+          <t>Radhakrishnan_Keerthi_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Radhakrishnan_Keerthi_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr"/>
@@ -3728,19 +3896,20 @@
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
       <c r="Q63" t="inlineStr"/>
-      <c r="R63" t="n">
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>9019s304b</t>
+          <t>j9602123n</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>10.18130/v3-m8p8-ad34</t>
+          <t>10.18130/v3-5rvv-6g36</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3748,30 +3917,32 @@
           <t>2020-05-06</t>
         </is>
       </c>
-      <c r="D64" t="n">
-        <v>4</v>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Karkar_Abhishek_Prospectus.pdf</t>
-        </is>
+      <c r="D64" s="2" t="n">
+        <v>44687</v>
+      </c>
+      <c r="E64" t="n">
+        <v>4</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Karkar_Abhishek_STS Research Paper.pdf</t>
+          <t>Tyree_Timothy_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Karkar_Abhishek_Sociotechnical Synthesis.pdf</t>
+          <t>Tyree_Timothy_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Karkar_Abhishek_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr"/>
+          <t>Tyree_Timothy_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Tyree_Timothy_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr"/>
@@ -3780,50 +3951,53 @@
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr"/>
       <c r="Q64" t="inlineStr"/>
-      <c r="R64" t="n">
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>3b5919181</t>
+          <t>zc77sq71p</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>10.18130/v3-zj6e-q755</t>
+          <t>10.18130/v3-pgc1-4e02</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2020-05-08</t>
-        </is>
-      </c>
-      <c r="D65" t="n">
-        <v>4</v>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Timmons_Eric_Prospectus.pdf</t>
-        </is>
+          <t>2020-05-07</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>45785</v>
+      </c>
+      <c r="E65" t="n">
+        <v>4</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Timmons_Eric_STS Research Paper.pdf</t>
+          <t>Kennedy_Jackson_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Timmons_Eric_Sociotechnical Synthesis.pdf</t>
+          <t>Kennedy_Jackson_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Timmons_Eric_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr"/>
+          <t>Kennedy_Jackson_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Kennedy_Jackson_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr"/>
@@ -3832,19 +4006,20 @@
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
       <c r="Q65" t="inlineStr"/>
-      <c r="R65" t="n">
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>xs55mc577</t>
+          <t>v692t682b</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>10.18130/v3-k063-3c17</t>
+          <t>10.18130/v3-8ytb-jw35</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3852,30 +4027,30 @@
           <t>2020-05-07</t>
         </is>
       </c>
-      <c r="D66" t="n">
-        <v>4</v>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Nguyen_Julian_Prospectus.pdf</t>
-        </is>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="n">
+        <v>4</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Nguyen_Julian_STS Research Paper.pdf</t>
+          <t>Kaylor_Christopher_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Nguyen_Julian_Sociotechnical Synthesis.pdf</t>
+          <t>Kaylor_Christopher_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Nguyen_Julian_Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr"/>
+          <t>Kaylor_Christopher_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Kaylor_Christopher_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr"/>
@@ -3884,50 +4059,51 @@
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr"/>
       <c r="Q66" t="inlineStr"/>
-      <c r="R66" t="n">
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="n">
         <v>2020</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>x059c791g</t>
+          <t>s4655h213</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>10.18130/v3-kayq-sm25</t>
+          <t>10.18130/v3-w6qe-3f60</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2020-05-07</t>
-        </is>
-      </c>
-      <c r="D67" t="n">
-        <v>4</v>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Prospectus.pdf</t>
-        </is>
+          <t>2020-05-05</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="n">
+        <v>4</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>STS Research Paper.pdf</t>
+          <t>Gumabay_Ethan_Prospectus.pdf</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Sociotechnical Synthesis.pdf</t>
+          <t>Gumabay_Ethan_STS Research Paper.pdf</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Technical Report.pdf</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr"/>
+          <t>Gumabay_Ethan_Sociotechnical Synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Gumabay_Ethan_Technical Report.pdf</t>
+        </is>
+      </c>
       <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr"/>
@@ -3936,7 +4112,8 @@
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr"/>
       <c r="Q67" t="inlineStr"/>
-      <c r="R67" t="n">
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="n">
         <v>2020</v>
       </c>
     </row>

</xml_diff>